<commit_message>
added customer price & nationality
</commit_message>
<xml_diff>
--- a/assets/upload-sample/sample/Customer_Upload.xlsx
+++ b/assets/upload-sample/sample/Customer_Upload.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp-8.2.4\htdocs\off_pos\assets\upload-sample\sample\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\trul-salon\assets\upload-sample\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323AF19B-87ED-4E15-A252-D392C234B7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CF0C65-42AF-49FC-8563-4D20FA023008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Customer Bulk Upload</t>
   </si>
@@ -141,6 +141,12 @@
   </si>
   <si>
     <t>+88 0188888</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Nationality</t>
   </si>
 </sst>
 </file>
@@ -219,7 +225,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -242,9 +248,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -527,23 +530,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="24.85546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="25" style="3" customWidth="1"/>
-    <col min="5" max="5" width="27.140625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="43.7109375" style="6" customWidth="1"/>
-    <col min="7" max="7" width="39.85546875" style="6" customWidth="1"/>
-    <col min="8" max="8" width="32.5703125" customWidth="1"/>
-    <col min="9" max="9" width="40.28515625" customWidth="1"/>
-    <col min="10" max="10" width="24.85546875" style="7" customWidth="1"/>
-    <col min="11" max="11" width="36.85546875" style="7" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" customWidth="1"/>
+    <col min="2" max="3" width="24.88671875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="25" style="3" customWidth="1"/>
+    <col min="6" max="6" width="27.109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="43.6640625" style="6" customWidth="1"/>
+    <col min="8" max="8" width="39.88671875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="32.5546875" customWidth="1"/>
+    <col min="10" max="10" width="40.33203125" customWidth="1"/>
+    <col min="11" max="11" width="24.88671875" style="7" customWidth="1"/>
+    <col min="12" max="12" width="35.6640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -552,102 +555,111 @@
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
       <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="171.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="171.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>10</v>
       </c>
+      <c r="M3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <v>500</v>
       </c>
-      <c r="G4" s="6">
+      <c r="H4" s="6">
         <v>5</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>13</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="7">
+      <c r="K4" s="7">
         <v>45402</v>
       </c>
-      <c r="K4" s="7">
+      <c r="L4" s="7">
         <v>45402</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4" xr:uid="{67BE4999-7A36-4CBE-8D93-E88E38C80CC1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4" xr:uid="{67BE4999-7A36-4CBE-8D93-E88E38C80CC1}">
       <formula1>"Debit, Credit"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4" xr:uid="{4A1E66A9-FF42-471E-9F56-8C3766290A4E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4" xr:uid="{4A1E66A9-FF42-471E-9F56-8C3766290A4E}">
       <formula1>"Retail, Wholesale"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>

<commit_message>
added customer price & nationality (#15)
</commit_message>
<xml_diff>
--- a/assets/upload-sample/sample/Customer_Upload.xlsx
+++ b/assets/upload-sample/sample/Customer_Upload.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp-8.2.4\htdocs\off_pos\assets\upload-sample\sample\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\trul-salon\assets\upload-sample\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323AF19B-87ED-4E15-A252-D392C234B7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CF0C65-42AF-49FC-8563-4D20FA023008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Customer Bulk Upload</t>
   </si>
@@ -141,6 +141,12 @@
   </si>
   <si>
     <t>+88 0188888</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Nationality</t>
   </si>
 </sst>
 </file>
@@ -219,7 +225,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -242,9 +248,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -527,23 +530,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
-    <col min="2" max="2" width="24.85546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="25" style="3" customWidth="1"/>
-    <col min="5" max="5" width="27.140625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="43.7109375" style="6" customWidth="1"/>
-    <col min="7" max="7" width="39.85546875" style="6" customWidth="1"/>
-    <col min="8" max="8" width="32.5703125" customWidth="1"/>
-    <col min="9" max="9" width="40.28515625" customWidth="1"/>
-    <col min="10" max="10" width="24.85546875" style="7" customWidth="1"/>
-    <col min="11" max="11" width="36.85546875" style="7" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" customWidth="1"/>
+    <col min="2" max="3" width="24.88671875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="25" style="3" customWidth="1"/>
+    <col min="6" max="6" width="27.109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="43.6640625" style="6" customWidth="1"/>
+    <col min="8" max="8" width="39.88671875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="32.5546875" customWidth="1"/>
+    <col min="10" max="10" width="40.33203125" customWidth="1"/>
+    <col min="11" max="11" width="24.88671875" style="7" customWidth="1"/>
+    <col min="12" max="12" width="35.6640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -552,102 +555,111 @@
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
       <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
-    <row r="2" spans="1:11" ht="171.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="171.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>10</v>
       </c>
+      <c r="M3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <v>500</v>
       </c>
-      <c r="G4" s="6">
+      <c r="H4" s="6">
         <v>5</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>13</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="7">
+      <c r="K4" s="7">
         <v>45402</v>
       </c>
-      <c r="K4" s="7">
+      <c r="L4" s="7">
         <v>45402</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4" xr:uid="{67BE4999-7A36-4CBE-8D93-E88E38C80CC1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4" xr:uid="{67BE4999-7A36-4CBE-8D93-E88E38C80CC1}">
       <formula1>"Debit, Credit"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4" xr:uid="{4A1E66A9-FF42-471E-9F56-8C3766290A4E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4" xr:uid="{4A1E66A9-FF42-471E-9F56-8C3766290A4E}">
       <formula1>"Retail, Wholesale"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>